<commit_message>
feat(products): nuevas opciones de concentracion en form e importador
Actualiza el tipo, la lista de opciones y los alias del importador Excel
(EDP/EDT/EDC/ELIXIR/PARFUM/EXTRAIT/INTENSE). Plantillas xlsx regeneradas
con la nueva lista cerrada.
</commit_message>
<xml_diff>
--- a/public/plantilla-productos.xlsx
+++ b/public/plantilla-productos.xlsx
@@ -587,7 +587,7 @@
         <v>NOCHE</v>
       </c>
       <c r="Q2" t="str">
-        <v>ELIXIR_DE_PARFUM</v>
+        <v>ELIXIR</v>
       </c>
       <c r="R2" t="str">
         <v>ALTA</v>
@@ -932,7 +932,7 @@
         <v>no</v>
       </c>
       <c r="D20" t="str">
-        <v>EAU_DE_PARFUM · EAU_DE_TOILETTE · ELIXIR_DE_PARFUM · EAU_DE_COLOGNE · BODY_MIST · PARFUM_EXTRAIT (acepta EDP/EDT/EDC/EXTRAIT)</v>
+        <v>EAU_DE_PARFUM · EAU_DE_TOILETTE · EAU_DE_TOILETTE_INTENSE · EAU_DE_COLOGNE · BODY_MIST · ELIXIR · PARFUM · EXTRAIT_DE_PARFUM (acepta EDP/EDT/EDC/ELIXIR/PARFUM/EXTRAIT/INTENSE)</v>
       </c>
     </row>
     <row r="21">

</xml_diff>